<commit_message>
Remove old Streamlit app/ folder, add update_log.py
The Streamlit-based app/ directory has been replaced by the Dash rewrite
in dash_app/. Removes all old app/ files from tracking and adds update_log.py.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NN_Design_Tracker.xlsx
+++ b/NN_Design_Tracker.xlsx
@@ -3210,7 +3210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3526,6 +3526,31 @@
       <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Next: end-to-end test with MyRawdata.xlsx. A7 value=8 (NEE) custom missing handling still pending. Re-zip and upload to Google Drive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="200" customHeight="1">
+      <c r="A14" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Stage 0 column editor — drop columns reflect immediately on Apply changes</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Dash app startup verified — all dependencies installed (kaleido, diskcache, choreographer newly added). Bug fix in Stage 0 (Data Audit) column editor: previously, columns marked as Drop and applied via 'Apply changes' button remained visible in the AgGrid column editor with Drop=True, requiring manual visual inspection to confirm removal. Fix: (1) apply_changes callback now includes a third Output — s0-col-grid rowData — returning only kept rows with Drop reset to False, so dropped columns disappear from the grid immediately on button press. (2) flag_sweep callback updated with allow_duplicate=True on its s0-col-grid Output to avoid Dash duplicate output conflict. (3) layout() function updated to filter out previously-dropped columns (from _col_editor_prior state) when re-rendering Stage 0, so navigating away and back does not cause dropped columns to reappear in the editor.</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Test full Dash pipeline end-to-end with MyRawdata.xlsx + survey.docx. A7 value=8 (NEE) custom missing handling still pending. Re-zip and upload to Google Drive. Decide whether to keep Streamlit app as fallback or remove it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Variable Mapping redesign + sidebar collapse + Stage 0 upload fix
- var_mapping.py: full rewrite — accordion tile view groups columns by
  QNR question; each tile has type dropdown, move-to dropdown, delete
  button, and hover tooltip showing first 10 values + answer options;
  auto-detects possibly-related columns by prefix heuristic
- app.py: sidebar collapse toggle (hamburger button collapses to 48px,
  shifts content area); added sidebar-collapsed session store
- stage0_audit.py: replaced html.A with html.Span in upload area to
  prevent page refresh on click
- style.css: added vm-accordion, vm-q-code, vm-q-text, sidebar toggle styles
- update_log.py / NN_Design_Tracker.xlsx: sessions 14 & 15 logged

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NN_Design_Tracker.xlsx
+++ b/NN_Design_Tracker.xlsx
@@ -3210,7 +3210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3551,6 +3551,81 @@
       <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Test full Dash pipeline end-to-end with MyRawdata.xlsx + survey.docx. A7 value=8 (NEE) custom missing handling still pending. Re-zip and upload to Google Drive. Decide whether to keep Streamlit app as fallback or remove it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="200" customHeight="1">
+      <c r="A15" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Git cleanup (removed Streamlit app/) + Stage 0 upload fix + debug mode off</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Session 2026-04-10 changes: (1) Git repo cleanup on branch dash-app: removed old Streamlit app/ directory (18 files) from git tracking via 'git rm', staged update_log.py and updated NN_Design_Tracker.xlsx, committed as '93376bd — Remove old Streamlit app/ folder, add update_log.py', pushed to origin/dash-app. The Streamlit app/ has been fully replaced by the Dash rewrite in dash_app/. (2) Bug fix — Stage 0 CSV upload caused full page refresh: the dcc.Upload children contained html.A('click to select') with no href, which some browsers treat as a page navigation/reload. Fixed by replacing html.A with html.Span (same styling). (3) Removed debug=True from app.run() — set to debug=False to suppress the Plotly/Dash debug toolbar and 'install Plotly cloud' prompt that appeared on every page load.</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Test full Dash pipeline end-to-end with MyRawdata.xlsx + survey.docx. A7 value=8 (NEE) custom missing handling still pending. Re-zip and upload to Google Drive. Continue logging all code changes in update_log.py per session.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="200" customHeight="1">
+      <c r="A16" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Variable Mapping redesign — accordion tiles, hover preview, delete/move, sidebar collapse</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Session 2026-04-10 — Variable Mapping page full redesign: (1) Replaced flat AgGrid table with accordion tile view — each QNR question is a collapsible card; each dataset column is a tile showing column name, type dropdown, 'Move to question' dropdown, and delete (X) button. (2) Hover tooltip on column name shows first 10 non-null values, unique/missing counts, and QNR answer options. (3) 'Possibly related' columns detected automatically — columns whose prefix starts with a question code but with an alphabetic suffix (e.g. A6B related to A6) shown in amber tiles inside that question's card. (4) Reassign/move: changing the 'Move to question' dropdown reassigns a column to a different question group. (5) Delete: X button removes a column from the mapping view; 'Reset all' restores deleted/reassigned columns. (6) Summary row shows Active Columns, Questions Matched, Possibly Related, No QNR Match, QNR Only, Deleted counts. (7) Sidebar collapse toggle added — hamburger button always visible; clicking collapses sidebar to 48px icon strip and shifts content area for full-width workspace. State persists in session storage. (8) Fixed html.A browse links to html.Span in upload areas of var_mapping.py (same fix as stage0).</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Test accordion tile view with actual MyRawdata.xlsx + survey.docx. A7 value=8 (NEE) custom missing handling still pending. Re-zip and upload to Google Drive. Continue logging all code changes in update_log.py per session.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="200" customHeight="1">
+      <c r="A17" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Variable Mapping redesign — accordion tiles, hover preview, delete/move, sidebar collapse</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Session 2026-04-10 — Variable Mapping page full redesign: (1) Replaced flat AgGrid table with accordion tile view — each QNR question is a collapsible card; each dataset column is a tile showing column name, type dropdown, 'Move to question' dropdown, and delete (X) button. (2) Hover tooltip on column name shows first 10 non-null values, unique/missing counts, and QNR answer options. (3) 'Possibly related' columns detected automatically — columns whose prefix starts with a question code but with an alphabetic suffix (e.g. A6B related to A6) shown in amber tiles inside that question's card. (4) Reassign/move: changing the 'Move to question' dropdown reassigns a column to a different question group. (5) Delete: X button removes a column from the mapping view; 'Reset all' restores deleted/reassigned columns. (6) Summary row shows Active Columns, Questions Matched, Possibly Related, No QNR Match, QNR Only, Deleted counts. (7) Sidebar collapse toggle added — hamburger button always visible; clicking collapses sidebar to 48px icon strip and shifts content area for full-width workspace. State persists in session storage. (8) Fixed html.A browse links to html.Span in upload areas of var_mapping.py (same fix as stage0).</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Test accordion tile view with actual MyRawdata.xlsx + survey.docx. A7 value=8 (NEE) custom missing handling still pending. Re-zip and upload to Google Drive. Continue logging all code changes in update_log.py per session.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inline options per tile + docx table-order fix in qnr_parser
- var_mapping.py: options moved into each tile as pill chips (max 6 +
  overflow count); scale questions show low/high anchors; removed
  card-level options panel; _render_tile gains scale_str parameter
- qnr_parser.py: _parse_docx rewritten to iterate doc.element.body in
  document order so tables immediately following a question are parsed
  as its options; handles single-cell, value|label, and multi-cell rows;
  merged cells deduplicated by element identity
- CLAUDE.md: updated to session 16 with tile/parser details
- update_log.py / NN_Design_Tracker.xlsx: session 16 logged

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NN_Design_Tracker.xlsx
+++ b/NN_Design_Tracker.xlsx
@@ -3210,7 +3210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3626,6 +3626,31 @@
       <c r="E17" s="4" t="inlineStr">
         <is>
           <t>Test accordion tile view with actual MyRawdata.xlsx + survey.docx. A7 value=8 (NEE) custom missing handling still pending. Re-zip and upload to Google Drive. Continue logging all code changes in update_log.py per session.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="200" customHeight="1">
+      <c r="A18" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Var Mapping: inline options per tile + qnr_parser docx table-order fix</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Session 2026-04-10 (continued) — Variable Mapping further improvements: (1) Answer options moved from card-level panel into each individual variable tile — each tile now shows its question's options as indigo pill chips (max 6 visible + '+N more'). Scale questions show '1 = low → N = high' anchor text instead. (2) qnr_parser.py _parse_docx rewritten to read docx in true document order (paragraphs and tables interleaved). Previously all paragraphs were read first then all tables, breaking the question→options link when options live in Word tables. Fix uses doc.element.body iteration with qn('w:p') / qn('w:tbl') tags. Handles three table layouts: single-cell rows (one option per row), two-cell value|label rows (formats as '1. Label'), and multi-cell rows (joined with ' | '). Merged cells deduplicated by element identity.</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Test full pipeline end-to-end with MyRawdata.xlsx + survey.docx. A7 value=8 (NEE) custom missing handling still pending. Re-zip and upload to Google Drive. Continue logging all code changes in update_log.py per session.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Session 17 log: Var Mapping interactive option assignment
Updated update_log.py, NN_Design_Tracker.xlsx (session 17 row), and
CLAUDE.md current state to reflect the multi-select option assignment
feature added to variable tiles.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NN_Design_Tracker.xlsx
+++ b/NN_Design_Tracker.xlsx
@@ -3210,7 +3210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3649,6 +3649,31 @@
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Test full pipeline end-to-end with MyRawdata.xlsx + survey.docx. A7 value=8 (NEE) custom missing handling still pending. Re-zip and upload to Google Drive. Continue logging all code changes in update_log.py per session.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="200" customHeight="1">
+      <c r="A19" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Var Mapping: interactive multi-select option assignment per variable tile</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Session 2026-04-10 — Var Mapping: interactive option assignment per variable tile. Replaced static read-only answer-option chips on each variable tile with an interactive multi-select dropdown. Each tile now shows an 'Assigned options' dropdown populated with the parent question's answer options from the QNR; user can select one or more options to indicate which answer options that variable represents. Selections stored in vm_state['option_assignments'] (dict: col -&gt; list of selected option strings) and persist within the session. Reset all clears assignments along with other vm_state fields. Callback: handle_option_assign uses pattern-matching Input({'type': 'vm-opt-sel', 'index': ALL}). DEFAULT_VM_STATE updated to include 'option_assignments': {}. Committed as 4f8dea8 and pushed to origin/dash-app.</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>Test full pipeline end-to-end with MyRawdata.xlsx + survey.docx. A7 value=8 (NEE) custom missing handling still pending. Re-zip and upload to Google Drive. Continue logging all code changes in update_log.py per session.</t>
         </is>

</xml_diff>

<commit_message>
Session 18: Var Mapping table+drag-drop redesign + QC fixes
- var_mapping: replace accordion tiles with 4-col table per question
  (Variable | Options | Type | Question); options as draggable chips
- assets/dragdrop.js: new — document-level drag-and-drop handler
- assets/style.css: opt-chip, opt-dropzone, pool styles added
- Auto-assignment: single col→all opts, multi+suffix→indexed opt,
  grid→all opts, scale/numeric→no chips; unassigned pool row
- Save button: clientside_callback reads DOM → vm-drag-assignments
  store → handle_save commits all changes at once
- vm-state: storage_type memory→session (survives navigation)
- handle_save: guard empty drag_assigns to protect saved assignments
- stage0_audit: remove duplicate s0-upload-status component ID
- app.py: render_page app-state State→Input (pages re-render on upload)
- CLAUDE.md + update_log + NN_Design_Tracker updated (session 18)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NN_Design_Tracker.xlsx
+++ b/NN_Design_Tracker.xlsx
@@ -3210,7 +3210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3676,6 +3676,31 @@
       <c r="E19" s="4" t="inlineStr">
         <is>
           <t>Test full pipeline end-to-end with MyRawdata.xlsx + survey.docx. A7 value=8 (NEE) custom missing handling still pending. Re-zip and upload to Google Drive. Continue logging all code changes in update_log.py per session.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="200" customHeight="1">
+      <c r="A20" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Var Mapping: table+drag-drop redesign; Stage 0 + app.py QC fixes</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Session 2026-04-10 — Var Mapping redesign + QC fixes. (1) Variable Mapping page fully redesigned: replaced per-variable accordion tiles with a 4-column table per question (Variable | Options | Type | Question). Options rendered as draggable HTML chips (opt-chip class); drag-and-drop handled by assets/dragdrop.js using document-level event delegation so listeners survive Dash re-renders. Drop zones (opt-dropzone) highlight on hover. Auto-assignment logic: single col → all opts; multi q_type + numeric/letter suffix → indexed opt; grid → all opts per col; scale/numeric → no chips. Unassigned options pool row shown at table bottom. Save button triggers clientside_callback that reads DOM chip positions into vm-drag-assignments store, then handle_save server callback commits all changes. vm-state storage changed to session so assignments survive page navigation. handle_save guards against empty drag_assigns dict overwriting saved option_assignments. (2) Stage 0 QC fix: removed duplicate id=s0-upload-status element (was at lines 103 and 159). (3) app.py QC fix: render_page app-state changed from State to Input so pages re-render immediately after upload without requiring navigation. New file: dash_app/assets/dragdrop.js. CSS additions: opt-chip, opt-dropzone, opt-chip-pool styles.</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Test full pipeline end-to-end with MyRawdata.xlsx + survey.docx. A7 value=8 (NEE) custom missing handling still pending. Re-zip and upload to Google Drive. Stages 1-9 inherited from Streamlit rewrite, not yet re-tested end-to-end.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Session 19: qnr_parser docx rewrite + grid-prefix expansion + B3 flush fix
- _parse_docx returns list[dict] directly via two-pass approach
- New _parse_table_for_options: skips merged rows (vMerge, gridSpan>1,
  single-cell disclaimers), reads first column only, stores
  table_col_headers and table_n_cols for downstream grid detection
- Table path: pre-table paragraphs → question text; table → options
- No-table path: last paragraph → single option
- Grid-prefix expansion in _default_option_assignments: expands options
  as 'col_header opt' when n_vars ≈ n_opts × (n_table_cols-1) ±10%
- Bug fix: flush called with [] instead of text_buf in had_table branch,
  silently discarding pre-table paragraphs (affected B3-type questions)
- CLAUDE.md and session log updated (session 19, row 21)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NN_Design_Tracker.xlsx
+++ b/NN_Design_Tracker.xlsx
@@ -3210,7 +3210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3699,6 +3699,31 @@
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Test full pipeline end-to-end with MyRawdata.xlsx + survey.docx. A7 value=8 (NEE) custom missing handling still pending. Re-zip and upload to Google Drive. Stages 1-9 inherited from Streamlit rewrite, not yet re-tested end-to-end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="200" customHeight="1">
+      <c r="A21" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>qnr_parser docx rewrite: proper merge detection, table-path/no-table-path, grid-prefix expansion, B3 flush bug fix</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Session 2026-04-17 — qnr_parser docx rewrite + var_mapping grid-prefix expansion + B3 flush bug fix. (1) _parse_docx fully rewritten to return list[dict] directly instead of list[str]. New _parse_table_for_options helper: skips row 0 always; reads ONLY first column; skips vertical-merge continuation rows (w:vMerge without val=restart); skips horizontally-merged first-cell rows (w:gridSpan &gt; 1); skips single-cell disclaimer rows; extracts table_col_headers (row 0 cols 1+) and table_n_cols. Two-pass approach: pass 1 collects (para, text) and (table, obj) in document order; pass 2 groups into questions. Table path: buffered paragraphs before table → question text, table → options. No-table path: all paragraphs except last → question text, last → single option (unless it starts with Please/Your answers or is all-caps section header). Validation warning printed if extracted options &lt; 90% of unmerged row count. parse_questionnaire short-circuits for .docx, returning _parse_docx result directly. PDF/xlsx/txt paths unchanged. (2) _default_option_assignments in var_mapping.py: added grid-prefix expansion. For questions with table_n_cols &gt; 2 and table_col_headers present, if n_matched_vars approximately equals n_opts × (n_table_cols - 1) within ±10%, expands options as 'col_header opt' for each option × each column header, assigned 1:1 to matched+extra cols. (3) Bug fix: _flush_question called with [] instead of text_buf when a post-table paragraph appeared before the next question code — pre-table paragraphs were silently discarded. Fixed by passing text_buf in the had_table branch (qnr_parser.py line ~336).</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>Test full pipeline end-to-end with MyRawdata.xlsx + survey.docx. A7 value=8 (NEE) custom missing handling still pending. Re-zip and upload to Google Drive. Stages 1-9 inherited from Streamlit rewrite, not yet re-tested end-to-end.</t>
         </is>

</xml_diff>

<commit_message>
Session 20: Excel metadata auto-mapping for Var Mapping page
- col_mapper.py: parse_excel_metadata() reads 'Variable Label Information'
  and 'Value Label Information' sheets from data Excel (accepts path or BytesIO)
- col_mapper.py: build_questions_from_metadata() builds question dicts from
  those sheets — single-col uses value labels as chips, multi-col uses stripped
  column labels (one chip per column)
- var_mapping.py: upload_data callback auto-detects metadata sheets on xlsx
  upload, builds and stores questions immediately (no separate QNR upload needed)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NN_Design_Tracker.xlsx
+++ b/NN_Design_Tracker.xlsx
@@ -3210,7 +3210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3726,6 +3726,56 @@
       <c r="E21" s="4" t="inlineStr">
         <is>
           <t>Test full pipeline end-to-end with MyRawdata.xlsx + survey.docx. A7 value=8 (NEE) custom missing handling still pending. Re-zip and upload to Google Drive. Stages 1-9 inherited from Streamlit rewrite, not yet re-tested end-to-end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="200" customHeight="1">
+      <c r="A22" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>qnr_parser docx rewrite: proper merge detection, table-path/no-table-path, grid-prefix expansion, B3 flush bug fix</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Session 2026-04-17 — qnr_parser docx rewrite + var_mapping grid-prefix expansion + B3 flush bug fix. (1) _parse_docx fully rewritten to return list[dict] directly instead of list[str]. New _parse_table_for_options helper: skips row 0 always; reads ONLY first column; skips vertical-merge continuation rows (w:vMerge without val=restart); skips horizontally-merged first-cell rows (w:gridSpan &gt; 1); skips single-cell disclaimer rows; extracts table_col_headers (row 0 cols 1+) and table_n_cols. Two-pass approach: pass 1 collects (para, text) and (table, obj) in document order; pass 2 groups into questions. Table path: buffered paragraphs before table → question text, table → options. No-table path: all paragraphs except last → question text, last → single option (unless it starts with Please/Your answers or is all-caps section header). Validation warning printed if extracted options &lt; 90% of unmerged row count. parse_questionnaire short-circuits for .docx, returning _parse_docx result directly. PDF/xlsx/txt paths unchanged. (2) _default_option_assignments in var_mapping.py: added grid-prefix expansion. For questions with table_n_cols &gt; 2 and table_col_headers present, if n_matched_vars approximately equals n_opts × (n_table_cols - 1) within ±10%, expands options as 'col_header opt' for each option × each column header, assigned 1:1 to matched+extra cols. (3) Bug fix: _flush_question called with [] instead of text_buf when a post-table paragraph appeared before the next question code — pre-table paragraphs were silently discarded. Fixed by passing text_buf in the had_table branch (qnr_parser.py line ~336).</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Test full pipeline end-to-end with MyRawdata.xlsx + survey.docx. A7 value=8 (NEE) custom missing handling still pending. Re-zip and upload to Google Drive. Stages 1-9 inherited from Streamlit rewrite, not yet re-tested end-to-end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="200" customHeight="1">
+      <c r="A23" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-17 S20</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Excel metadata auto-mapping: parse_excel_metadata + build_questions_from_metadata in col_mapper.py; upload_data auto-detects Variable/Value Label sheets</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Session 2026-04-17 — Excel metadata auto-mapping for Variable Mapping page. Added two new functions to col_mapper.py: (1) parse_excel_metadata(source): reads 'Variable Label Information' and 'Value Label Information' sheets from a data Excel file (accepts file path or BytesIO). Returns var_labels dict {col_name: label_text} and value_labels dict {col_name: {numeric_value: label_str}}. Returns has_metadata=False if sheets absent. (2) build_questions_from_metadata(var_labels, value_labels, col_groups): builds question dicts in the same format as qnr_parser output. Single-column groups: options come from value_labels sorted by numeric key. Multi-column groups (multi/grid/multi_col): options come from stripped var_labels of each column (one chip per column, 'CODE - ' prefix removed). Type inferred from number of options and value key structure. Also added _CODE_STRIP_RE regex and _vl_sort_key helper. var_mapping.py upload_data callback updated: after loading the DataFrame, if file is xlsx/xls, calls parse_excel_metadata on the raw decoded bytes (BytesIO). If has_metadata=True, calls build_questions_from_metadata and stores result as qnr_questions in server_store, sets mapping_done=True immediately (no separate QNR upload needed). Status message appended with auto-mapped question count. Raw data 2.xlsx pulled from git remote: has 703 var_labels, 375 value_labels, builds 76 questions from 'Data with Values' sheet column groups.</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Test full pipeline end-to-end with Raw data 2.xlsx + Survey 2.docx. A7 value=8 (NEE) custom missing handling still pending. Type inference for single-col questions may misclassify categorical as scale_N (e.g. S1 with 7 options → scale_7); user can override on mapping page. Re-zip and upload to Google Drive. Stages 1-9 inherited from Streamlit rewrite, not yet re-tested end-to-end.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Session 21: Accurate variable-to-option assignment via QNR+Excel merge
- merge_qnr_with_metadata: intersection rule (QNR text canonical when overlap
  ≥40% word match), QNR-only when no overlap, no duplicate option versions
- Grid expansion: n_vars == n_opts × n_col_headers triggers prefix expansion;
  three detection modes (QNR headers, suffix-inferred, legacy table_n_cols>2)
- Zero-unassigned guarantee: suffix positional fallback then overassign all opts
- parse_excel_metadata: reads col B (var_types), case-insensitive sheet lookup
- _col_b_to_var_type helper; meta_var_type drives Type dropdown default
- refresh_mapping calls merge when both QNR and Excel metadata loaded
- _mapping_source annotation + DEBUG-level assignment logging per column
- CLAUDE.md and session log updated (session 21)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NN_Design_Tracker.xlsx
+++ b/NN_Design_Tracker.xlsx
@@ -3210,7 +3210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3776,6 +3776,31 @@
       <c r="E23" s="4" t="inlineStr">
         <is>
           <t>Test full pipeline end-to-end with Raw data 2.xlsx + Survey 2.docx. A7 value=8 (NEE) custom missing handling still pending. Type inference for single-col questions may misclassify categorical as scale_N (e.g. S1 with 7 options → scale_7); user can override on mapping page. Re-zip and upload to Google Drive. Stages 1-9 inherited from Streamlit rewrite, not yet re-tested end-to-end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="200" customHeight="1">
+      <c r="A24" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-20 S21</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Var Mapping: accurate option assignment via QNR+Excel merge — intersection rule, grid expansion, zero-unassigned safety pass, col-B type, debug logging</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Session 2026-04-20 — Accurate variable-to-option assignment using Excel metadata + QNR. col_mapper.py: parse_excel_metadata now reads col B (variable type) into var_types dict and uses case-insensitive sheet name lookup. Added _col_b_to_var_type() helper mapping raw col-B strings to canonical var-type keys. Added merge_qnr_with_metadata(questions, meta, col_groups) as the central enrichment function. Logic: (1) for each question, collect col-E labels from 'Variable Label Information' sheet for all matched columns; (2) test for overlap between QNR options and col-E labels using substring containment and word-overlap ratio &gt;= 0.4; (3) if overlap found → use INTERSECTION only, preserving QNR text as canonical (no duplicate option versions); if no overlap → use QNR options only; (4) grid expansion fires when n_matched_vars == n_options * n_col_headers, in three detection modes: QNR-provided table_col_headers, headers inferred from variable name suffixes, legacy table_n_cols &gt; 2; expanded options formatted as '{col_header} {option}' assigned sequentially; (5) safety pass ensures every column gets an assignment — suffix positional fallback (_1 → opts[0]) then overassign all options if still unresolved; (6) annotates each enriched question with _mapping_source and _mapping_warnings for auditability; (7) calls log_assignments() at DEBUG level for per-column assignment tracing. var_mapping.py: _default_option_assignments reordered so col_assignments branch runs before scale/numeric short-circuit (metadata assignments survive for all q_types); grid expansion block generalised to fire on col_headers length match, not just table_n_cols &gt; 2; final safety pass added after all loops to guarantee no column is left blank. refresh_mapping callback now calls merge_qnr_with_metadata when both QNR and Excel metadata are loaded. Type dropdown now prefers meta_var_type (col B) over heuristic suggest_var_type. Test result: 351 columns enriched, 0 unassigned across all matched questions.</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>S10B (and similar suffixed variants like S10b_N_1) not parsed from QNR docx — parser stops at S10A; these fall back to Excel metadata only. QNR parser fix pending. A7 value=8 (NEE) custom missing handling still pending (Stage 1). Test full pipeline end-to-end with Raw data 2.xlsx + survey.docx. Re-zip and upload to Google Drive. Stages 1-9 inherited from Streamlit rewrite, not yet re-tested end-to-end.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Session 22: QNR parse cross-validation — warn when option count < dataset columns
- col_mapper.py: Step 4b in merge_qnr_with_metadata() compares len(final_opts)
  against dataset column count / n_col_headers; emits log.warning + appends to
  _mapping_warnings when QNR options are <70% of expected (surfaces S10B-class bugs)
- var_mapping.py: red 'incomplete parse' badge in accordion header + inline alert
  block in accordion body for any question with the parse-incomplete warning
- Survey 2.docx updated by user
- Raw data 2.xlsx updated
- update_log.py + NN_Design_Tracker.xlsx: session 22 logged

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NN_Design_Tracker.xlsx
+++ b/NN_Design_Tracker.xlsx
@@ -3210,7 +3210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3801,6 +3801,31 @@
       <c r="E24" s="4" t="inlineStr">
         <is>
           <t>S10B (and similar suffixed variants like S10b_N_1) not parsed from QNR docx — parser stops at S10A; these fall back to Excel metadata only. QNR parser fix pending. A7 value=8 (NEE) custom missing handling still pending (Stage 1). Test full pipeline end-to-end with Raw data 2.xlsx + survey.docx. Re-zip and upload to Google Drive. Stages 1-9 inherited from Streamlit rewrite, not yet re-tested end-to-end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="200" customHeight="1">
+      <c r="A25" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-23 S22</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>QNR parse accuracy: Strategy 3 cross-validation — col_mapper warns when option count &lt; dataset column count; red badge + alert in Var Mapping UI</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Session 2026-04-23 — QNR parse accuracy: Strategy 3 cross-validation + incomplete-parse warning in UI. col_mapper.py: added Step 4b cross-validation block in merge_qnr_with_metadata(). After final_opts is settled and grid expansion has been attempted, compares len(final_opts) against len(dataset_cols) / n_col_headers. If QNR options are less than 70% of what the column count implies (and expected &gt; n_opts), appends a warning to _mapping_warnings AND emits log.warning() so it surfaces in the terminal without requiring DEBUG logging. Warning text format: '{CODE}: QNR has {n} option(s) but {m} dataset column(s) suggest ~{expected} — QNR parsing may be incomplete (check table structure in the source document)'. var_mapping.py: accordion card header now shows a red '⚠ incomplete parse' dbc.Badge for any question whose _mapping_warnings contains the parse-incomplete signal; badge title tooltip shows the full message. Inside the accordion body, a red inline alert box (background #fef2f2, border #fca5a5) renders the full warning text so the user sees the mismatch count without hovering. Survey 2.docx updated by user (re-uploaded). Raw data 2.xlsx updated (minor binary change).</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>S10B root cause still unknown — strategy 3 will now surface the exact mismatch count when Survey 2.docx + Raw data 2.xlsx are loaded in the app. Investigate the actual QNR docx structure for S10B once warning fires: check whether it is a page-break split table (Strategy 1) or vMerge skip on rows 10-20 (Strategy 2). A7 value=8 (NEE) custom missing value handling still pending (Stage 1). Test full pipeline end-to-end with Raw data 2.xlsx + Survey 2.docx. Re-zip and upload to Google Drive. Stages 1-9 inherited from Streamlit rewrite, not yet re-tested end-to-end.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Session 23 log: update_log.py + tracker entry
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NN_Design_Tracker.xlsx
+++ b/NN_Design_Tracker.xlsx
@@ -3210,7 +3210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3826,6 +3826,56 @@
       <c r="E25" s="4" t="inlineStr">
         <is>
           <t>S10B root cause still unknown — strategy 3 will now surface the exact mismatch count when Survey 2.docx + Raw data 2.xlsx are loaded in the app. Investigate the actual QNR docx structure for S10B once warning fires: check whether it is a page-break split table (Strategy 1) or vMerge skip on rows 10-20 (Strategy 2). A7 value=8 (NEE) custom missing value handling still pending (Stage 1). Test full pipeline end-to-end with Raw data 2.xlsx + Survey 2.docx. Re-zip and upload to Google Drive. Stages 1-9 inherited from Streamlit rewrite, not yet re-tested end-to-end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="200" customHeight="1">
+      <c r="A26" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-23 S22</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>QNR parse accuracy: Strategy 3 cross-validation — col_mapper warns when option count &lt; dataset column count; red badge + alert in Var Mapping UI</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Session 2026-04-23 — QNR parse accuracy: Strategy 3 cross-validation + incomplete-parse warning in UI. col_mapper.py: added Step 4b cross-validation block in merge_qnr_with_metadata(). After final_opts is settled and grid expansion has been attempted, compares len(final_opts) against len(dataset_cols) / n_col_headers. If QNR options are less than 70% of what the column count implies (and expected &gt; n_opts), appends a warning to _mapping_warnings AND emits log.warning() so it surfaces in the terminal without requiring DEBUG logging. Warning text format: '{CODE}: QNR has {n} option(s) but {m} dataset column(s) suggest ~{expected} — QNR parsing may be incomplete (check table structure in the source document)'. var_mapping.py: accordion card header now shows a red '⚠ incomplete parse' dbc.Badge for any question whose _mapping_warnings contains the parse-incomplete signal; badge title tooltip shows the full message. Inside the accordion body, a red inline alert box (background #fef2f2, border #fca5a5) renders the full warning text so the user sees the mismatch count without hovering. Survey 2.docx updated by user (re-uploaded). Raw data 2.xlsx updated (minor binary change).</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>S10B root cause still unknown — strategy 3 will now surface the exact mismatch count when Survey 2.docx + Raw data 2.xlsx are loaded in the app. Investigate the actual QNR docx structure for S10B once warning fires: check whether it is a page-break split table (Strategy 1) or vMerge skip on rows 10-20 (Strategy 2). A7 value=8 (NEE) custom missing value handling still pending (Stage 1). Test full pipeline end-to-end with Raw data 2.xlsx + Survey 2.docx. Re-zip and upload to Google Drive. Stages 1-9 inherited from Streamlit rewrite, not yet re-tested end-to-end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="200" customHeight="1">
+      <c r="A27" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-23 S23</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Fix S10B option truncation + import-options UI — overlap score fix, page-break table merge, borrowed-options auto-detect, Import from / Add to pool callbacks</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Session 2026-04-23 — Fix S10B option truncation + import-options UI. col_mapper.py: fixed _overlap_score substring collision where short tokens like 'p1' matched inside 'p10', 'p11' etc., causing intersection to drop options 10+. Changed containment check to word-boundary (set subset) instead of character substring. Removed early-exit at score&gt;=1.0 in _best_qnr_match so all options are compared; on equal score, prefer the longer/more specific QNR option. qnr_parser.py: merge continuation tables split across Word page breaks — when a second w:tbl element is encountered for the same question, its options are appended rather than silently dropped (had_table guard relaxed). Added _cell_is_blue() helper to detect blue-coloured font runs in a table cell. In _parse_table_for_options, row 1 col 0 is checked: if it is a short question code in blue text it is stored as borrows_options_from; after full-document dedup pass, questions with borrows_options_from and no options get the source question's options copied in. var_mapping.py: pool row now shows an 'Import from...' dcc.Dropdown listing all other question codes; selecting one runs import_options_from_question callback which appends source question's options into vm_state['extra_options'][target_code]. Textarea '+ Add / paste options' panel wired to server: add_options_to_pool callback reads one-per-line text and saves to extra_options. Both mechanisms deduplicate and persist across page navigation. DEFAULT_VM_STATE updated to include extra_options: {}. Pool construction in _render_var_table includes extra_options deduped with q['options'].</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>A7 value=8 (NEE) custom missing value handling still pending (Stage 1). Test full pipeline end-to-end with Raw data 2.xlsx + Survey 2.docx. Re-zip and upload to Google Drive. Stages 1-9 inherited from Streamlit rewrite, not yet re-tested end-to-end. borrows_options_from auto-detection from blue PN notes not yet verified against real survey docx — test with Survey 2.docx to confirm blue-text detection works.</t>
         </is>
       </c>
     </row>

</xml_diff>